<commit_message>
refactor: actualizar PDF paths y  mejora de extraccion de pagina
</commit_message>
<xml_diff>
--- a/docs/informe_ocr.xlsx
+++ b/docs/informe_ocr.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdc7d18634725e34/DIEGO/Proyectos TrustSystems/ocr-albaran/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdc7d18634725e34/DIEGO/Proyectos TrustSystems/ocr-albaran/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_2F2C762FE43395E42EA4004BF54727498384CC45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAB11C03-A9D5-4340-AFAC-56A337CB62EF}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="11_2F2C762FE43395E42EA4004BF54727498384CC45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A028D7D-1B6E-4C69-A355-C67217E6C220}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Informe OCR" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="68">
   <si>
     <t>archivo</t>
   </si>
@@ -154,12 +154,6 @@
     <t>ERROR</t>
   </si>
   <si>
-    <t>timeout of 600000ms exceeded</t>
-  </si>
-  <si>
-    <t>600.13</t>
-  </si>
-  <si>
     <t>EJEMPLO 4.pdf</t>
   </si>
   <si>
@@ -197,6 +191,39 @@
   </si>
   <si>
     <t>Comentario</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>No se encontró</t>
+  </si>
+  <si>
+    <t>Los albaranes vienen en distintos angulos, iluminación, calidad, zoom-in y zoom-out. Por más que se intente con distintas librerias de preproceso, hay demasiadas variables, no hay un formato determinista que permita resultados exitosos sin una IA especializada en estas tareas</t>
+  </si>
+  <si>
+    <t>Este es el ejemplo perfecto, todos los albaranes vienen en el mismo formato, no falló y lo obtuvo en cuestión de dos minutos</t>
+  </si>
+  <si>
+    <t>Baja calidad, documento muy alejado de la cámara</t>
+  </si>
+  <si>
+    <t>Formato ideal</t>
+  </si>
+  <si>
+    <t>Mucho ruido, muy alejado de la cámara. Un algoritmo que calcule el acercamiento necesario sería demasiado complejo porque siempre tiende a cambair el formato, el zoom, la iluminación, el ruido y demás variables</t>
+  </si>
+  <si>
+    <t>Demasiado alejado y aparte dos documentos en la misma página</t>
+  </si>
+  <si>
+    <t>Formato ideal, suficiente zoom, un documento por página, ruido casi nulo</t>
+  </si>
+  <si>
+    <t>Dos documentos por página</t>
+  </si>
+  <si>
+    <t>Demasiado ruido en la imagen del albaran</t>
   </si>
 </sst>
 </file>
@@ -271,7 +298,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -322,11 +349,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -408,6 +459,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -720,7 +780,8 @@
     <col min="1" max="1" width="28.109375" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="19.109375" style="2" customWidth="1"/>
     <col min="6" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.5546875" bestFit="1" customWidth="1"/>
@@ -728,7 +789,7 @@
     <col min="12" max="12" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="23.77734375" style="37" customWidth="1"/>
     <col min="14" max="14" width="18.88671875" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="15" max="15" width="51.88671875" style="37" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -774,8 +835,8 @@
       <c r="N1" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="10" t="s">
-        <v>58</v>
+      <c r="O1" s="33" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -813,7 +874,7 @@
       <c r="N2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="3"/>
+      <c r="O2" s="34"/>
     </row>
     <row r="3" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -858,7 +919,9 @@
       <c r="N3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="O3" s="3"/>
+      <c r="O3" s="34" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -897,7 +960,9 @@
       <c r="N4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="O4" s="3"/>
+      <c r="O4" s="34" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -936,9 +1001,11 @@
       <c r="N5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="O5" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>34</v>
       </c>
@@ -981,7 +1048,9 @@
       <c r="N6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="O6" s="3"/>
+      <c r="O6" s="34" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="7" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="22" t="s">
@@ -1026,7 +1095,7 @@
       <c r="N7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="O7" s="3"/>
+      <c r="O7" s="34"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
@@ -1065,7 +1134,9 @@
       <c r="N8" s="3">
         <v>399.51</v>
       </c>
-      <c r="O8" s="3"/>
+      <c r="O8" s="38" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -1104,7 +1175,7 @@
       <c r="N9" s="3">
         <v>399.51</v>
       </c>
-      <c r="O9" s="3"/>
+      <c r="O9" s="39"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -1143,7 +1214,7 @@
       <c r="N10" s="3">
         <v>399.51</v>
       </c>
-      <c r="O10" s="3"/>
+      <c r="O10" s="39"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -1182,7 +1253,7 @@
       <c r="N11" s="3">
         <v>399.51</v>
       </c>
-      <c r="O11" s="3"/>
+      <c r="O11" s="39"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
@@ -1221,7 +1292,7 @@
       <c r="N12" s="3">
         <v>399.51</v>
       </c>
-      <c r="O12" s="3"/>
+      <c r="O12" s="39"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -1260,7 +1331,7 @@
       <c r="N13" s="3">
         <v>399.51</v>
       </c>
-      <c r="O13" s="3"/>
+      <c r="O13" s="39"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
@@ -1299,7 +1370,7 @@
       <c r="N14" s="3">
         <v>399.51</v>
       </c>
-      <c r="O14" s="3"/>
+      <c r="O14" s="39"/>
     </row>
     <row r="15" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="22" t="s">
@@ -1338,56 +1409,58 @@
       <c r="N15" s="3">
         <v>399.51</v>
       </c>
-      <c r="O15" s="3"/>
-    </row>
-    <row r="16" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="O15" s="40"/>
+    </row>
+    <row r="16" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A16" s="18" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>43</v>
+        <v>24</v>
+      </c>
+      <c r="C16" s="27">
+        <v>56</v>
+      </c>
+      <c r="D16" s="27">
+        <v>0</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="H16" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="I16" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="J16" s="18" t="s">
-        <v>43</v>
+        <v>57</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="18" t="b">
+        <v>0</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="L16" s="18" t="s">
         <v>43</v>
       </c>
       <c r="M16" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="N16" s="3">
+        <v>1400</v>
+      </c>
+      <c r="O16" s="34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="O16" s="3"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>46</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
@@ -1418,13 +1491,15 @@
       <c r="L17" s="3"/>
       <c r="M17" s="34"/>
       <c r="N17" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="O17" s="3"/>
+        <v>45</v>
+      </c>
+      <c r="O17" s="34" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>15</v>
@@ -1445,7 +1520,7 @@
         <v>2551029785</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I18" s="9">
         <v>226.8</v>
@@ -1459,11 +1534,11 @@
       <c r="N18" s="3">
         <v>122.73</v>
       </c>
-      <c r="O18" s="3"/>
-    </row>
-    <row r="19" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O18" s="34"/>
+    </row>
+    <row r="19" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>15</v>
@@ -1496,11 +1571,13 @@
       <c r="N19" s="3">
         <v>146.22</v>
       </c>
-      <c r="O19" s="3"/>
+      <c r="O19" s="34" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="20" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>15</v>
@@ -1521,7 +1598,7 @@
         <v>8351008553</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I20" s="30">
         <v>7.74</v>
@@ -1539,11 +1616,13 @@
       <c r="N20" s="3">
         <v>211.29</v>
       </c>
-      <c r="O20" s="3"/>
+      <c r="O20" s="38" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="21" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>15</v>
@@ -1557,14 +1636,14 @@
       <c r="E21" s="9">
         <v>18</v>
       </c>
-      <c r="F21" s="13" t="s">
-        <v>16</v>
+      <c r="F21" s="12">
+        <v>95</v>
       </c>
       <c r="G21" s="12">
         <v>8351008554</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I21" s="9">
         <v>8.8000000000000007</v>
@@ -1584,11 +1663,11 @@
       <c r="N21" s="3">
         <v>211.29</v>
       </c>
-      <c r="O21" s="3"/>
+      <c r="O21" s="39"/>
     </row>
     <row r="22" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>15</v>
@@ -1609,7 +1688,7 @@
         <v>8351008552</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I22" s="9">
         <v>1055.24</v>
@@ -1627,11 +1706,11 @@
       <c r="N22" s="3">
         <v>211.29</v>
       </c>
-      <c r="O22" s="3"/>
+      <c r="O22" s="39"/>
     </row>
     <row r="23" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B23" s="22" t="s">
         <v>15</v>
@@ -1652,7 +1731,7 @@
         <v>9051006723</v>
       </c>
       <c r="H23" s="25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I23" s="32">
         <v>8.8699999999999992</v>
@@ -1670,11 +1749,11 @@
       <c r="N23" s="3">
         <v>211.29</v>
       </c>
-      <c r="O23" s="3"/>
+      <c r="O23" s="40"/>
     </row>
     <row r="24" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>15</v>
@@ -1715,11 +1794,13 @@
       <c r="N24" s="3">
         <v>42.4</v>
       </c>
-      <c r="O24" s="3"/>
+      <c r="O24" s="37" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>15</v>
@@ -1752,9 +1833,15 @@
       <c r="N25" s="3">
         <v>295.42</v>
       </c>
-      <c r="O25" s="3"/>
+      <c r="O25" s="34" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="O8:O15"/>
+    <mergeCell ref="O20:O23"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: agregar excepción quick-OCR para páginas casi en blanco en el procesamiento de PDFs
</commit_message>
<xml_diff>
--- a/docs/informe_ocr.xlsx
+++ b/docs/informe_ocr.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdc7d18634725e34/DIEGO/Proyectos TrustSystems/ocr-albaran/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djlop\OneDrive\DIEGO\Proyectos TrustSystems\ocr-albaran\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="11_2F2C762FE43395E42EA4004BF54727498384CC45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A028D7D-1B6E-4C69-A355-C67217E6C220}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FB0A0F1-A9D6-4000-B7B1-A67C91D84ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Informe OCR" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="67">
   <si>
     <t>archivo</t>
   </si>
@@ -149,9 +149,6 @@
   </si>
   <si>
     <t>EJEMPLO 3.pdf</t>
-  </si>
-  <si>
-    <t>ERROR</t>
   </si>
   <si>
     <t>EJEMPLO 4.pdf</t>
@@ -836,10 +833,10 @@
         <v>13</v>
       </c>
       <c r="O1" s="33" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -876,7 +873,7 @@
       </c>
       <c r="O2" s="34"/>
     </row>
-    <row r="3" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>18</v>
       </c>
@@ -920,10 +917,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="34" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
@@ -961,10 +958,10 @@
         <v>29</v>
       </c>
       <c r="O4" s="34" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
@@ -1002,10 +999,10 @@
         <v>33</v>
       </c>
       <c r="O5" s="34" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>34</v>
       </c>
@@ -1049,7 +1046,7 @@
         <v>35</v>
       </c>
       <c r="O6" s="34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1135,7 +1132,7 @@
         <v>399.51</v>
       </c>
       <c r="O8" s="38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1425,42 +1422,42 @@
         <v>0</v>
       </c>
       <c r="E16" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K16" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="36" t="s">
-        <v>58</v>
-      </c>
       <c r="L16" s="18" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="M16" s="36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N16" s="3">
         <v>1400</v>
       </c>
       <c r="O16" s="34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
@@ -1491,15 +1488,15 @@
       <c r="L17" s="3"/>
       <c r="M17" s="34"/>
       <c r="N17" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O17" s="34" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>15</v>
@@ -1520,7 +1517,7 @@
         <v>2551029785</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I18" s="9">
         <v>226.8</v>
@@ -1532,13 +1529,13 @@
       <c r="L18" s="3"/>
       <c r="M18" s="34"/>
       <c r="N18" s="3">
-        <v>122.73</v>
+        <v>31.52</v>
       </c>
       <c r="O18" s="34"/>
     </row>
     <row r="19" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>15</v>
@@ -1572,12 +1569,12 @@
         <v>146.22</v>
       </c>
       <c r="O19" s="34" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>15</v>
@@ -1598,7 +1595,7 @@
         <v>8351008553</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I20" s="30">
         <v>7.74</v>
@@ -1617,12 +1614,12 @@
         <v>211.29</v>
       </c>
       <c r="O20" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>15</v>
@@ -1643,7 +1640,7 @@
         <v>8351008554</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I21" s="9">
         <v>8.8000000000000007</v>
@@ -1667,7 +1664,7 @@
     </row>
     <row r="22" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>15</v>
@@ -1688,7 +1685,7 @@
         <v>8351008552</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I22" s="9">
         <v>1055.24</v>
@@ -1710,7 +1707,7 @@
     </row>
     <row r="23" spans="1:15" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" s="22" t="s">
         <v>15</v>
@@ -1731,7 +1728,7 @@
         <v>9051006723</v>
       </c>
       <c r="H23" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I23" s="32">
         <v>8.8699999999999992</v>
@@ -1751,9 +1748,9 @@
       </c>
       <c r="O23" s="40"/>
     </row>
-    <row r="24" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>15</v>
@@ -1795,12 +1792,12 @@
         <v>42.4</v>
       </c>
       <c r="O24" s="37" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>15</v>
@@ -1834,7 +1831,7 @@
         <v>295.42</v>
       </c>
       <c r="O25" s="34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>